<commit_message>
Updated YAML comments and text, fixed positive test case error and negative test case validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000672/negative/01/data/unit-test-coreid-FB3901-negative.xlsx
+++ b/rules/CORE-000672/negative/01/data/unit-test-coreid-FB3901-negative.xlsx
@@ -1,11 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
@@ -13,35 +9,62 @@
     <sheet name="lb.xpt" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -51,19 +74,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF9E"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,48 +106,33 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -264,6 +279,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -298,6 +314,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -332,20 +349,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -467,7 +480,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -482,24 +534,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>sendig</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
@@ -520,24 +572,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>lb.xpt</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Laboratory Test Results</t>
         </is>
@@ -554,39 +606,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Error group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Error level</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Row num</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Error value</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>LBTESTCD</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>CHOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRLO</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRHI</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>LBTESTCD</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>CHOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRLO</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRHI</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>LBTESTCD</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>HBA1CHGB</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRLO</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>LBSTNRHI</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -751,391 +1047,391 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Pool Identifier</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Sponsor-Defined Identifier</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Lab Test or Examination Short Name</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Lab Test or Examination Name</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Category for Lab Test</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>Reference Range Lower Limit in Orig Unit</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>Reference Range Upper Limit in Orig Unit</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>Specimen</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>Character Result/Finding in Std Format</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>Numeric Result/Finding in Standard Units</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>Standard Units</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>Reference Range Lower Limit-Std Units</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>Reference Range Upper Limit-Std Units</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="T2" s="7" t="inlineStr">
         <is>
           <t>Reference Range Indicator</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="U2" s="7" t="inlineStr">
         <is>
           <t>LOINC Code</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="V2" s="7" t="inlineStr">
         <is>
           <t>Specimen Type</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="W2" s="7" t="inlineStr">
         <is>
           <t>Derived Flag</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="X2" s="7" t="inlineStr">
         <is>
           <t>Baseline Flag</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Y2" s="7" t="inlineStr">
         <is>
           <t>Epoch</t>
         </is>
       </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="Z2" s="7" t="inlineStr">
         <is>
           <t>Visit Number</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
+      <c r="AA2" s="7" t="inlineStr">
         <is>
           <t>Visit Name</t>
         </is>
       </c>
-      <c r="AB2" s="4" t="inlineStr">
+      <c r="AB2" s="7" t="inlineStr">
         <is>
           <t>Date/Time of Specimen Collection</t>
         </is>
       </c>
-      <c r="AC2" s="4" t="inlineStr">
+      <c r="AC2" s="7" t="inlineStr">
         <is>
           <t>Study Day of Specimen Collection</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="R3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="S3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="T3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
+      <c r="V3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="W3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="X3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr">
+      <c r="Y3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="Z3" s="4" t="inlineStr">
+      <c r="Z3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="inlineStr">
+      <c r="AA3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="AB3" s="4" t="inlineStr">
+      <c r="AB3" s="7" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="AC3" s="4" t="inlineStr">
+      <c r="AC3" s="7" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U4" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="V4" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="W4" s="4" t="inlineStr">
+      <c r="W4" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X4" s="4" t="n">
+      <c r="X4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="4" t="n">
+      <c r="Y4" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="Z4" s="4" t="n">
+      <c r="Z4" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="AA4" s="4" t="n">
+      <c r="AA4" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="AB4" s="4" t="n">
+      <c r="AB4" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="AC4" s="4" t="n">
+      <c r="AC4" s="7" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1155,7 +1451,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n"/>
+      <c r="D5" s="5" t="str"/>
       <c r="E5" s="5" t="n">
         <v>1</v>
       </c>
@@ -1189,8 +1485,8 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
+      <c r="L5" s="5" t="str"/>
+      <c r="M5" s="5" t="str"/>
       <c r="N5" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1209,9 +1505,9 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
+      <c r="R5" s="5" t="str"/>
+      <c r="S5" s="5" t="str"/>
+      <c r="T5" s="5" t="str"/>
       <c r="U5" s="5" t="inlineStr">
         <is>
           <t>1751-7</t>
@@ -1222,8 +1518,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W5" s="5" t="n"/>
-      <c r="X5" s="5" t="n"/>
+      <c r="W5" s="5" t="str"/>
+      <c r="X5" s="5" t="str"/>
       <c r="Y5" s="5" t="inlineStr">
         <is>
           <t>SCREENING</t>
@@ -1262,7 +1558,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
+      <c r="D6" s="5" t="str"/>
       <c r="E6" s="5" t="n">
         <v>2</v>
       </c>
@@ -1296,8 +1592,8 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
+      <c r="L6" s="5" t="str"/>
+      <c r="M6" s="5" t="str"/>
       <c r="N6" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1326,7 +1622,7 @@
           <t>8.0</t>
         </is>
       </c>
-      <c r="T6" s="5" t="n"/>
+      <c r="T6" s="5" t="str"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
           <t>1751-7</t>
@@ -1337,8 +1633,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W6" s="5" t="n"/>
-      <c r="X6" s="5" t="n"/>
+      <c r="W6" s="5" t="str"/>
+      <c r="X6" s="5" t="str"/>
       <c r="Y6" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -1377,7 +1673,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
+      <c r="D7" s="5" t="str"/>
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
@@ -1411,8 +1707,8 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
+      <c r="L7" s="5" t="str"/>
+      <c r="M7" s="5" t="str"/>
       <c r="N7" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1431,9 +1727,9 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
+      <c r="R7" s="5" t="str"/>
+      <c r="S7" s="5" t="str"/>
+      <c r="T7" s="5" t="str"/>
       <c r="U7" s="5" t="inlineStr">
         <is>
           <t>1751-7</t>
@@ -1444,8 +1740,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="5" t="n"/>
+      <c r="W7" s="5" t="str"/>
+      <c r="X7" s="5" t="str"/>
       <c r="Y7" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -1484,7 +1780,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
+      <c r="D8" s="5" t="str"/>
       <c r="E8" s="5" t="n">
         <v>4</v>
       </c>
@@ -1518,8 +1814,8 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
+      <c r="L8" s="5" t="str"/>
+      <c r="M8" s="5" t="str"/>
       <c r="N8" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1538,9 +1834,9 @@
           <t>g/dL</t>
         </is>
       </c>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
-      <c r="T8" s="5" t="n"/>
+      <c r="R8" s="5" t="str"/>
+      <c r="S8" s="5" t="str"/>
+      <c r="T8" s="5" t="str"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
           <t>1751-7</t>
@@ -1551,8 +1847,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="5" t="n"/>
+      <c r="W8" s="5" t="str"/>
+      <c r="X8" s="5" t="str"/>
       <c r="Y8" s="5" t="inlineStr">
         <is>
           <t>FOLLOW-UP</t>
@@ -1591,7 +1887,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="5" t="str"/>
       <c r="E9" s="5" t="n">
         <v>5</v>
       </c>
@@ -1625,8 +1921,8 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
+      <c r="L9" s="5" t="str"/>
+      <c r="M9" s="5" t="str"/>
       <c r="N9" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1655,7 +1951,7 @@
           <t>21.5</t>
         </is>
       </c>
-      <c r="T9" s="5" t="n"/>
+      <c r="T9" s="5" t="str"/>
       <c r="U9" s="5" t="inlineStr">
         <is>
           <t>1742-6</t>
@@ -1666,8 +1962,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W9" s="5" t="n"/>
-      <c r="X9" s="5" t="n"/>
+      <c r="W9" s="5" t="str"/>
+      <c r="X9" s="5" t="str"/>
       <c r="Y9" s="5" t="inlineStr">
         <is>
           <t>SCREENING</t>
@@ -1706,7 +2002,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="5" t="str"/>
       <c r="E10" s="5" t="n">
         <v>6</v>
       </c>
@@ -1740,8 +2036,8 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="L10" s="5" t="str"/>
+      <c r="M10" s="5" t="str"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1760,9 +2056,9 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
+      <c r="R10" s="5" t="str"/>
+      <c r="S10" s="5" t="str"/>
+      <c r="T10" s="5" t="str"/>
       <c r="U10" s="5" t="inlineStr">
         <is>
           <t>1742-6</t>
@@ -1773,8 +2069,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W10" s="5" t="n"/>
-      <c r="X10" s="5" t="n"/>
+      <c r="W10" s="5" t="str"/>
+      <c r="X10" s="5" t="str"/>
       <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -1813,7 +2109,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="5" t="str"/>
       <c r="E11" s="5" t="n">
         <v>7</v>
       </c>
@@ -1847,8 +2143,8 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="L11" s="5" t="str"/>
+      <c r="M11" s="5" t="str"/>
       <c r="N11" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1867,9 +2163,9 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="R11" s="5" t="n"/>
-      <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
+      <c r="R11" s="5" t="str"/>
+      <c r="S11" s="5" t="str"/>
+      <c r="T11" s="5" t="str"/>
       <c r="U11" s="5" t="inlineStr">
         <is>
           <t>1742-6</t>
@@ -1880,8 +2176,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W11" s="5" t="n"/>
-      <c r="X11" s="5" t="n"/>
+      <c r="W11" s="5" t="str"/>
+      <c r="X11" s="5" t="str"/>
       <c r="Y11" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -1920,7 +2216,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n"/>
+      <c r="D12" s="5" t="str"/>
       <c r="E12" s="5" t="n">
         <v>8</v>
       </c>
@@ -1954,8 +2250,8 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
+      <c r="L12" s="5" t="str"/>
+      <c r="M12" s="5" t="str"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -1974,9 +2270,9 @@
           <t>U/L</t>
         </is>
       </c>
-      <c r="R12" s="5" t="n"/>
-      <c r="S12" s="5" t="n"/>
-      <c r="T12" s="5" t="n"/>
+      <c r="R12" s="5" t="str"/>
+      <c r="S12" s="5" t="str"/>
+      <c r="T12" s="5" t="str"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
           <t>1742-6</t>
@@ -1987,8 +2283,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W12" s="5" t="n"/>
-      <c r="X12" s="5" t="n"/>
+      <c r="W12" s="5" t="str"/>
+      <c r="X12" s="5" t="str"/>
       <c r="Y12" s="5" t="inlineStr">
         <is>
           <t>FOLLOW-UP</t>
@@ -2027,7 +2323,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="5" t="str"/>
       <c r="E13" s="5" t="n">
         <v>9</v>
       </c>
@@ -2036,7 +2332,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>CHOL</t>
         </is>
@@ -2061,8 +2357,8 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
+      <c r="L13" s="5" t="str"/>
+      <c r="M13" s="5" t="str"/>
       <c r="N13" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2081,17 +2377,17 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="R13" s="6" t="inlineStr">
+      <c r="R13" s="8" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
+      <c r="S13" s="9" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="T13" s="5" t="n"/>
+      <c r="T13" s="5" t="str"/>
       <c r="U13" s="5" t="inlineStr">
         <is>
           <t>2093-3</t>
@@ -2102,8 +2398,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W13" s="5" t="n"/>
-      <c r="X13" s="5" t="n"/>
+      <c r="W13" s="5" t="str"/>
+      <c r="X13" s="5" t="str"/>
       <c r="Y13" s="5" t="inlineStr">
         <is>
           <t>SCREENING</t>
@@ -2142,7 +2438,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
+      <c r="D14" s="5" t="str"/>
       <c r="E14" s="5" t="n">
         <v>10</v>
       </c>
@@ -2151,7 +2447,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>CHOL</t>
         </is>
@@ -2176,8 +2472,8 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
+      <c r="L14" s="5" t="str"/>
+      <c r="M14" s="5" t="str"/>
       <c r="N14" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2196,17 +2492,17 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="R14" s="7" t="inlineStr">
+      <c r="R14" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="S14" s="7" t="inlineStr">
+      <c r="S14" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="T14" s="5" t="n"/>
+      <c r="T14" s="5" t="str"/>
       <c r="U14" s="5" t="inlineStr">
         <is>
           <t>2093-3</t>
@@ -2217,8 +2513,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" s="5" t="n"/>
+      <c r="W14" s="5" t="str"/>
+      <c r="X14" s="5" t="str"/>
       <c r="Y14" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -2257,7 +2553,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n"/>
+      <c r="D15" s="5" t="str"/>
       <c r="E15" s="5" t="n">
         <v>11</v>
       </c>
@@ -2291,8 +2587,8 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
+      <c r="L15" s="5" t="str"/>
+      <c r="M15" s="5" t="str"/>
       <c r="N15" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2311,9 +2607,9 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="R15" s="5" t="n"/>
-      <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
+      <c r="R15" s="5" t="str"/>
+      <c r="S15" s="5" t="str"/>
+      <c r="T15" s="5" t="str"/>
       <c r="U15" s="5" t="inlineStr">
         <is>
           <t>2093-3</t>
@@ -2324,8 +2620,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W15" s="5" t="n"/>
-      <c r="X15" s="5" t="n"/>
+      <c r="W15" s="5" t="str"/>
+      <c r="X15" s="5" t="str"/>
       <c r="Y15" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -2364,7 +2660,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n"/>
+      <c r="D16" s="5" t="str"/>
       <c r="E16" s="5" t="n">
         <v>12</v>
       </c>
@@ -2398,8 +2694,8 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
+      <c r="L16" s="5" t="str"/>
+      <c r="M16" s="5" t="str"/>
       <c r="N16" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2418,9 +2714,9 @@
           <t>mmol/L</t>
         </is>
       </c>
-      <c r="R16" s="5" t="n"/>
-      <c r="S16" s="5" t="n"/>
-      <c r="T16" s="5" t="n"/>
+      <c r="R16" s="5" t="str"/>
+      <c r="S16" s="5" t="str"/>
+      <c r="T16" s="5" t="str"/>
       <c r="U16" s="5" t="inlineStr">
         <is>
           <t>2093-3</t>
@@ -2431,8 +2727,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W16" s="5" t="n"/>
-      <c r="X16" s="5" t="n"/>
+      <c r="W16" s="5" t="str"/>
+      <c r="X16" s="5" t="str"/>
       <c r="Y16" s="5" t="inlineStr">
         <is>
           <t>FOLLOW-UP</t>
@@ -2471,7 +2767,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n"/>
+      <c r="D17" s="5" t="str"/>
       <c r="E17" s="5" t="n">
         <v>13</v>
       </c>
@@ -2505,8 +2801,8 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
+      <c r="L17" s="5" t="str"/>
+      <c r="M17" s="5" t="str"/>
       <c r="N17" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2525,9 +2821,9 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="R17" s="5" t="n"/>
-      <c r="S17" s="5" t="n"/>
-      <c r="T17" s="5" t="n"/>
+      <c r="R17" s="5" t="str"/>
+      <c r="S17" s="5" t="str"/>
+      <c r="T17" s="5" t="str"/>
       <c r="U17" s="5" t="inlineStr">
         <is>
           <t>14682-9</t>
@@ -2538,8 +2834,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W17" s="5" t="n"/>
-      <c r="X17" s="5" t="n"/>
+      <c r="W17" s="5" t="str"/>
+      <c r="X17" s="5" t="str"/>
       <c r="Y17" s="5" t="inlineStr">
         <is>
           <t>SCREENING</t>
@@ -2578,7 +2874,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n"/>
+      <c r="D18" s="5" t="str"/>
       <c r="E18" s="5" t="n">
         <v>14</v>
       </c>
@@ -2612,8 +2908,8 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="5" t="n"/>
+      <c r="L18" s="5" t="str"/>
+      <c r="M18" s="5" t="str"/>
       <c r="N18" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2632,9 +2928,9 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="R18" s="5" t="n"/>
-      <c r="S18" s="5" t="n"/>
-      <c r="T18" s="5" t="n"/>
+      <c r="R18" s="5" t="str"/>
+      <c r="S18" s="5" t="str"/>
+      <c r="T18" s="5" t="str"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
           <t>14682-9</t>
@@ -2645,8 +2941,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W18" s="5" t="n"/>
-      <c r="X18" s="5" t="n"/>
+      <c r="W18" s="5" t="str"/>
+      <c r="X18" s="5" t="str"/>
       <c r="Y18" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -2685,7 +2981,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n"/>
+      <c r="D19" s="5" t="str"/>
       <c r="E19" s="5" t="n">
         <v>15</v>
       </c>
@@ -2719,8 +3015,8 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
+      <c r="L19" s="5" t="str"/>
+      <c r="M19" s="5" t="str"/>
       <c r="N19" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2739,9 +3035,9 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="R19" s="5" t="n"/>
-      <c r="S19" s="5" t="n"/>
-      <c r="T19" s="5" t="n"/>
+      <c r="R19" s="5" t="str"/>
+      <c r="S19" s="5" t="str"/>
+      <c r="T19" s="5" t="str"/>
       <c r="U19" s="5" t="inlineStr">
         <is>
           <t>14682-9</t>
@@ -2752,8 +3048,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W19" s="5" t="n"/>
-      <c r="X19" s="5" t="n"/>
+      <c r="W19" s="5" t="str"/>
+      <c r="X19" s="5" t="str"/>
       <c r="Y19" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -2792,7 +3088,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n"/>
+      <c r="D20" s="5" t="str"/>
       <c r="E20" s="5" t="n">
         <v>16</v>
       </c>
@@ -2826,8 +3122,8 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="L20" s="5" t="n"/>
-      <c r="M20" s="5" t="n"/>
+      <c r="L20" s="5" t="str"/>
+      <c r="M20" s="5" t="str"/>
       <c r="N20" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2846,9 +3142,9 @@
           <t>umol/L</t>
         </is>
       </c>
-      <c r="R20" s="5" t="n"/>
-      <c r="S20" s="5" t="n"/>
-      <c r="T20" s="5" t="n"/>
+      <c r="R20" s="5" t="str"/>
+      <c r="S20" s="5" t="str"/>
+      <c r="T20" s="5" t="str"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
           <t>14682-9</t>
@@ -2859,8 +3155,8 @@
           <t>SERUM</t>
         </is>
       </c>
-      <c r="W20" s="5" t="n"/>
-      <c r="X20" s="5" t="n"/>
+      <c r="W20" s="5" t="str"/>
+      <c r="X20" s="5" t="str"/>
       <c r="Y20" s="5" t="inlineStr">
         <is>
           <t>FOLLOW-UP</t>
@@ -2899,7 +3195,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n"/>
+      <c r="D21" s="5" t="str"/>
       <c r="E21" s="5" t="n">
         <v>17</v>
       </c>
@@ -2908,7 +3204,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>HBA1CHGB</t>
         </is>
@@ -2933,8 +3229,8 @@
           <t>mmol/mol</t>
         </is>
       </c>
-      <c r="L21" s="5" t="n"/>
-      <c r="M21" s="5" t="n"/>
+      <c r="L21" s="5" t="str"/>
+      <c r="M21" s="5" t="str"/>
       <c r="N21" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -2953,17 +3249,17 @@
           <t>mmol/mol</t>
         </is>
       </c>
-      <c r="R21" s="7" t="inlineStr">
+      <c r="R21" s="9" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="S21" s="7" t="inlineStr">
+      <c r="S21" s="9" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="T21" s="5" t="n"/>
+      <c r="T21" s="5" t="str"/>
       <c r="U21" s="5" t="inlineStr">
         <is>
           <t>59261-8</t>
@@ -2974,8 +3270,8 @@
           <t>BLOOD</t>
         </is>
       </c>
-      <c r="W21" s="5" t="n"/>
-      <c r="X21" s="5" t="n"/>
+      <c r="W21" s="5" t="str"/>
+      <c r="X21" s="5" t="str"/>
       <c r="Y21" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>
@@ -3014,7 +3310,7 @@
           <t>CDISC-TEST-001</t>
         </is>
       </c>
-      <c r="D22" s="5" t="n"/>
+      <c r="D22" s="5" t="str"/>
       <c r="E22" s="5" t="n">
         <v>18</v>
       </c>
@@ -3048,8 +3344,8 @@
           <t>mmol/mol</t>
         </is>
       </c>
-      <c r="L22" s="5" t="n"/>
-      <c r="M22" s="5" t="n"/>
+      <c r="L22" s="5" t="str"/>
+      <c r="M22" s="5" t="str"/>
       <c r="N22" s="5" t="inlineStr">
         <is>
           <t>BLOOD</t>
@@ -3068,9 +3364,9 @@
           <t>mmol/mol</t>
         </is>
       </c>
-      <c r="R22" s="5" t="n"/>
-      <c r="S22" s="5" t="n"/>
-      <c r="T22" s="5" t="n"/>
+      <c r="R22" s="5" t="str"/>
+      <c r="S22" s="5" t="str"/>
+      <c r="T22" s="5" t="str"/>
       <c r="U22" s="5" t="inlineStr">
         <is>
           <t>59261-8</t>
@@ -3081,8 +3377,8 @@
           <t>BLOOD</t>
         </is>
       </c>
-      <c r="W22" s="5" t="n"/>
-      <c r="X22" s="5" t="n"/>
+      <c r="W22" s="5" t="str"/>
+      <c r="X22" s="5" t="str"/>
       <c r="Y22" s="5" t="inlineStr">
         <is>
           <t>TREATMENT</t>

</xml_diff>